<commit_message>
feat: add standalone Meta WhatsApp automation and optimize Render deployment
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\Desktop\Whatapp Messaging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A740E422-0E1A-4BA5-860B-F94D420DDB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A30E48-C043-4815-AC7F-259F67B6BA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Numbers" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>phone</t>
   </si>
@@ -37,130 +37,28 @@
     <t>error</t>
   </si>
   <si>
-    <t>966555508674</t>
-  </si>
-  <si>
     <t>تويوتا كامري GLE 2022</t>
   </si>
   <si>
     <t>https://haraj.com.sa/11184538452/</t>
   </si>
   <si>
-    <t>966557770796</t>
-  </si>
-  <si>
     <t>برادو 2007</t>
   </si>
   <si>
     <t>https://haraj.com.sa/11184538436/</t>
   </si>
   <si>
-    <t>966559680177</t>
-  </si>
-  <si>
     <t>تيوتاء كامري 2019</t>
   </si>
   <si>
     <t>https://haraj.com.sa/11184538424/</t>
   </si>
   <si>
-    <t>966565008037</t>
-  </si>
-  <si>
     <t>كامري 2022 GLE هايبرد</t>
   </si>
   <si>
     <t>https://haraj.com.sa/11184538397/</t>
-  </si>
-  <si>
-    <t>966579727232</t>
-  </si>
-  <si>
-    <t>هايلكس 2022</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184538370/</t>
-  </si>
-  <si>
-    <t>966547551527</t>
-  </si>
-  <si>
-    <t>لاندكروزر للبيع</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184538401/</t>
-  </si>
-  <si>
-    <t>966554662922</t>
-  </si>
-  <si>
-    <t>جيب لاند كروزر فكسار 1993</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542228/</t>
-  </si>
-  <si>
-    <t>966537039820</t>
-  </si>
-  <si>
-    <t>للبيع كامري موديل 14</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542224/</t>
-  </si>
-  <si>
-    <t>966509866911</t>
-  </si>
-  <si>
-    <t>كامري 2013 نظيفة</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542155/</t>
-  </si>
-  <si>
-    <t>966560606621</t>
-  </si>
-  <si>
-    <t>تويوتا هايلكس دبل ديزل 2022</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542152/</t>
-  </si>
-  <si>
-    <t>966503102710</t>
-  </si>
-  <si>
-    <t>اف جي 16</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542117/</t>
-  </si>
-  <si>
-    <t>966565262143</t>
-  </si>
-  <si>
-    <t>تويوتا فورتشنر 2023</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542100/</t>
-  </si>
-  <si>
-    <t>966508171169</t>
-  </si>
-  <si>
-    <t>تويوتا كامري 2014 GLX</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184542009/</t>
-  </si>
-  <si>
-    <t>966593123103</t>
-  </si>
-  <si>
-    <t>لاندكروزر VXR 2023 فل كامل</t>
-  </si>
-  <si>
-    <t>https://haraj.com.sa/11184541987/</t>
   </si>
   <si>
     <t>url</t>
@@ -447,13 +345,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.77734375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -461,7 +359,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -474,198 +372,58 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="4">
+        <v>201128247939</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>7</v>
       </c>
       <c r="D2" s="4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="4">
+        <v>201289996040</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="D3" s="4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
+      <c r="A4" s="4">
+        <v>201157765587</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D4" s="4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>14</v>
+      <c r="A5" s="4">
+        <v>201000056796</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D5" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="4" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>